<commit_message>
docs: fix typos in docstrings and comments
</commit_message>
<xml_diff>
--- a/HousePrices-AdvancedRegressionTechniques/notebooks/Performance_Comparison.xlsx
+++ b/HousePrices-AdvancedRegressionTechniques/notebooks/Performance_Comparison.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
     <t xml:space="preserve">Train</t>
   </si>
@@ -53,6 +53,9 @@
   </si>
   <si>
     <t xml:space="preserve">SVR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Performance comparison of models based on feature counts</t>
   </si>
 </sst>
 </file>
@@ -62,7 +65,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -98,6 +101,13 @@
       <family val="2"/>
       <charset val="1"/>
     </font>
+    <font>
+      <b val="true"/>
+      <sz val="12"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -141,7 +151,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -160,6 +170,10 @@
     </xf>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -715,149 +729,25 @@
         <v>0.222</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="18.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="0"/>
-      <c r="B12" s="0"/>
-      <c r="C12" s="0"/>
-      <c r="D12" s="0"/>
-      <c r="E12" s="0"/>
-      <c r="F12" s="0"/>
-      <c r="G12" s="0"/>
-      <c r="H12" s="0"/>
-      <c r="I12" s="0"/>
-      <c r="J12" s="0"/>
-      <c r="K12" s="0"/>
-      <c r="L12" s="0"/>
-      <c r="M12" s="0"/>
-      <c r="N12" s="0"/>
-      <c r="O12" s="0"/>
-      <c r="P12" s="0"/>
-    </row>
-    <row r="13" customFormat="false" ht="18.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="0"/>
-      <c r="B13" s="0"/>
-      <c r="C13" s="0"/>
-      <c r="D13" s="0"/>
-      <c r="E13" s="0"/>
-      <c r="F13" s="0"/>
-      <c r="G13" s="0"/>
-      <c r="H13" s="0"/>
-      <c r="I13" s="0"/>
-      <c r="J13" s="0"/>
-      <c r="K13" s="0"/>
-      <c r="L13" s="0"/>
-      <c r="M13" s="0"/>
-      <c r="N13" s="0"/>
-      <c r="O13" s="0"/>
-      <c r="P13" s="0"/>
-    </row>
-    <row r="14" customFormat="false" ht="18.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="0"/>
-      <c r="B14" s="0"/>
-      <c r="C14" s="0"/>
-      <c r="D14" s="0"/>
-      <c r="E14" s="0"/>
-      <c r="F14" s="0"/>
-      <c r="G14" s="0"/>
-      <c r="H14" s="0"/>
-      <c r="I14" s="0"/>
-      <c r="J14" s="0"/>
-      <c r="K14" s="0"/>
-      <c r="L14" s="0"/>
-      <c r="M14" s="0"/>
-      <c r="N14" s="0"/>
-      <c r="O14" s="0"/>
-      <c r="P14" s="0"/>
-    </row>
-    <row r="15" customFormat="false" ht="18.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="0"/>
-      <c r="B15" s="0"/>
-      <c r="C15" s="0"/>
-      <c r="D15" s="0"/>
-      <c r="E15" s="0"/>
-      <c r="F15" s="0"/>
-      <c r="G15" s="0"/>
-      <c r="H15" s="0"/>
-      <c r="I15" s="0"/>
-      <c r="J15" s="0"/>
-      <c r="K15" s="0"/>
-      <c r="L15" s="0"/>
-      <c r="M15" s="0"/>
-      <c r="N15" s="0"/>
-      <c r="O15" s="0"/>
-      <c r="P15" s="0"/>
-    </row>
-    <row r="16" customFormat="false" ht="18.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="0"/>
-      <c r="B16" s="0"/>
-      <c r="C16" s="0"/>
-      <c r="D16" s="0"/>
-      <c r="E16" s="0"/>
-      <c r="F16" s="0"/>
-      <c r="G16" s="0"/>
-      <c r="H16" s="0"/>
-      <c r="I16" s="0"/>
-      <c r="J16" s="0"/>
-      <c r="K16" s="0"/>
-      <c r="L16" s="0"/>
-      <c r="M16" s="0"/>
-      <c r="N16" s="0"/>
-      <c r="O16" s="0"/>
-      <c r="P16" s="0"/>
-    </row>
-    <row r="17" customFormat="false" ht="18.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="0"/>
-      <c r="B17" s="0"/>
-      <c r="C17" s="0"/>
-      <c r="D17" s="0"/>
-      <c r="E17" s="0"/>
-      <c r="F17" s="0"/>
-      <c r="G17" s="0"/>
-      <c r="H17" s="0"/>
-      <c r="I17" s="0"/>
-      <c r="J17" s="0"/>
-      <c r="K17" s="0"/>
-      <c r="L17" s="0"/>
-      <c r="M17" s="0"/>
-      <c r="N17" s="0"/>
-      <c r="O17" s="0"/>
-      <c r="P17" s="0"/>
-    </row>
-    <row r="18" customFormat="false" ht="18.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="0"/>
-      <c r="B18" s="0"/>
-      <c r="C18" s="0"/>
-      <c r="D18" s="0"/>
-      <c r="E18" s="0"/>
-      <c r="F18" s="0"/>
-      <c r="G18" s="0"/>
-      <c r="H18" s="0"/>
-      <c r="I18" s="0"/>
-      <c r="J18" s="0"/>
-      <c r="K18" s="0"/>
-      <c r="L18" s="0"/>
-      <c r="M18" s="0"/>
-      <c r="N18" s="0"/>
-      <c r="O18" s="0"/>
-      <c r="P18" s="0"/>
-    </row>
-    <row r="19" customFormat="false" ht="18.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="0"/>
-      <c r="B19" s="0"/>
-      <c r="C19" s="0"/>
-      <c r="D19" s="0"/>
-      <c r="E19" s="0"/>
-      <c r="F19" s="0"/>
-      <c r="G19" s="0"/>
-      <c r="H19" s="0"/>
-      <c r="I19" s="0"/>
-      <c r="J19" s="0"/>
-      <c r="K19" s="0"/>
-      <c r="L19" s="0"/>
-      <c r="M19" s="0"/>
-      <c r="N19" s="0"/>
-      <c r="O19" s="0"/>
-      <c r="P19" s="0"/>
+    <row r="10" customFormat="false" ht="18.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="B10" s="5"/>
+      <c r="C10" s="5"/>
+      <c r="D10" s="5"/>
+      <c r="E10" s="5"/>
+      <c r="F10" s="5"/>
+      <c r="G10" s="5"/>
+      <c r="H10" s="5"/>
+      <c r="I10" s="5"/>
+      <c r="J10" s="5"/>
+      <c r="K10" s="5"/>
+      <c r="L10" s="5"/>
+      <c r="M10" s="5"/>
+      <c r="N10" s="5"/>
+      <c r="O10" s="5"/>
+      <c r="P10" s="5"/>
     </row>
     <row r="20" customFormat="false" ht="18.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="2"/>
@@ -878,10 +768,11 @@
       <c r="P20" s="2"/>
     </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="4">
     <mergeCell ref="B1:F1"/>
     <mergeCell ref="G1:K1"/>
     <mergeCell ref="L1:P1"/>
+    <mergeCell ref="A10:P10"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.025" bottom="1.025" header="0.7875" footer="0.7875"/>

</xml_diff>